<commit_message>
Oppdaterer lister med 2026 H1-resultater og publiserer nettsideforbedringer.
Integrerer nye rådata, oppdaterer topplister og statistikk, og legger til siste innlagte registreringer med sortering og paginering på nettsiden.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/EndResult/100m Bryst.xlsx
+++ b/EndResult/100m Bryst.xlsx
@@ -646,25 +646,25 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Gabriel Rognes Steen</t>
+          <t>Ole Skuseth</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>1.06,93</t>
+          <t>1.06,68</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>563</v>
+        <v>569</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>01.12.2024</t>
+          <t>25.01.2026</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Vejle</t>
+          <t>Trondheim</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -681,25 +681,25 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Simen Løvås</t>
+          <t>Gabriel Rognes Steen</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>1.07,13</t>
+          <t>1.06,93</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>558</v>
+        <v>563</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>14.11.2021</t>
+          <t>01.12.2024</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Porsgrunn</t>
+          <t>Vejle</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -716,25 +716,25 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Sebastian Amundsen</t>
+          <t>Simen Løvås</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>1.07,72</t>
+          <t>1.07,13</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>543</v>
+        <v>558</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>17.01.2020</t>
+          <t>14.11.2021</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Trondheim</t>
+          <t>Porsgrunn</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -786,20 +786,20 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Ole Skuseth</t>
+          <t>Sebastian Amundsen</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>1.07,84</t>
+          <t>1.07,72</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>541</v>
+        <v>543</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>26.04.2025</t>
+          <t>17.01.2020</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -1047,25 +1047,25 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Ådne Viken Refseth</t>
+          <t>Einar Woldseth</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>1.10,11</t>
+          <t>1.09,91</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>533</v>
+        <v>538</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>16.07.2016</t>
+          <t>17.04.2026</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Kristiansand</t>
+          <t>Bergen</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -1082,25 +1082,25 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Gabriel Rognes Steen</t>
+          <t>Ole Skuseth</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>1.10,22</t>
+          <t>1.09,98</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>531</v>
+        <v>536</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>22.04.2024</t>
+          <t>17.04.2026</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Funchal</t>
+          <t>Bergen</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -1117,25 +1117,25 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Simen Løvås</t>
+          <t>Ådne Viken Refseth</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>1.10,39</t>
+          <t>1.10,11</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>527</v>
+        <v>533</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>01.04.2022</t>
+          <t>16.07.2016</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Bergen</t>
+          <t>Kristiansand</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -1152,25 +1152,25 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Johan Hjelseth Storstad</t>
+          <t>Gabriel Rognes Steen</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>1.11,02</t>
+          <t>1.10,22</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>513</v>
+        <v>531</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>05.07.2021</t>
+          <t>22.04.2024</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Bergen</t>
+          <t>Funchal</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -1187,25 +1187,25 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Sebastian Amundsen</t>
+          <t>Simen Løvås</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>1.11,06</t>
+          <t>1.10,39</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>512</v>
+        <v>527</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>15.06.2019</t>
+          <t>01.04.2022</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Hamar</t>
+          <t>Bergen</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -1483,20 +1483,20 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Stine Tveit</t>
+          <t>Sissel Furuholt Valle</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>1.15,25</t>
+          <t>1.14,74</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>569</v>
+        <v>580</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>22.01.2011</t>
+          <t>13.06.2026</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -1518,20 +1518,20 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Sara Alonso Lopez</t>
+          <t>Stine Tveit</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>1.15,36</t>
+          <t>1.15,25</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>566</v>
+        <v>569</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>15.01.2023</t>
+          <t>22.01.2011</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -1553,12 +1553,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Julie Mathilde Bjordal</t>
+          <t>Sara Alonso Lopez</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>1.15,35</t>
+          <t>1.15,36</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -1566,7 +1566,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>18.01.2019</t>
+          <t>15.01.2023</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -1588,25 +1588,25 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Sanna Josefin Husan Ehrnholm</t>
+          <t>Julie Mathilde Bjordal</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>1.15,76</t>
+          <t>1.15,35</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>557</v>
+        <v>566</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>26.10.2014</t>
+          <t>18.01.2019</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Kristiansund</t>
+          <t>Trondheim</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -1954,25 +1954,25 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Andrea Lintorp</t>
+          <t>Sissel Furuholt Valle</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>1.19,08</t>
+          <t>1.17,80</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>533</v>
+        <v>560</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>17.07.2014</t>
+          <t>02.07.2026</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Drammen</t>
+          <t>Tøyen</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -1989,20 +1989,20 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Stine Tveit</t>
+          <t>Andrea Lintorp</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>1.19,44</t>
+          <t>1.19,08</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>526</v>
+        <v>533</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>09.07.2011</t>
+          <t>17.07.2014</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">

</xml_diff>